<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.002-03 La guirlande d'anniversaire de Mila
Réécriture vocale example4 : éclat de tiroir, Nino reste assis, Mila s'assoit.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.002-03.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.002-03.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salle à manger le matin</t>
+          <t>salle à manger le matin, volets, tiroir de papiers, colle</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mila, Nino, papa</t>
+          <t>Mila, Nino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut une guirlande de papier pour l'anniversaire de papa. Nino arrive. Le corps n'est pas une blague. Un anneau se déchire. Ils allongent la guirlande, ensemble.</t>
+          <t>Le tiroir de papiers est entrouvert. Ça sent la colle. Les volets laissent un rai mince. Sur le bois, un éclat de tiroir luit. Mila veut une guirlande jusqu'à la fenêtre, maintenant, avec Nino. Elle tire trop vite : Nino reste assis, l'anneau se déchire. Sourire parti. Elle refuse de foncer, s'assoit, dit d'accord. Merci vécu. Elle tire vers le haut : la guirlande penche. Elle s'arrête, lit l'éclat. Un éclat de tiroir reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les volets laissent un rai de poussière d'or. Un tiroir de papiers est ouvert. Ça sent la colle, un peu sucré. Un fil pend du buffet. Une paire de ciseaux attend sur le bois. La chaise a un fil qui dépasse. Tu as vu le rai de soleil, Mila ? Il est tout fin. Oui. Il traverse la salle. En ce moment, Mila coupe un rectangle. Les ciseaux font un petit cri. Le papier est rouge et un peu rêche. C'est pour toi, papa. Une guirlande. Jusqu'à la fenêtre ? Oui. Tout le chemin. Nino arrive avec des chaussettes silencieuses. Nino a un corps plus rond. Mila a un corps plus mince. Mila ne commente pas le corps. Le corps n'est pas une blague. On joue. Nino, tu veux coller ? Oui. Ils collent le premier anneau. Le papier frotte entre les doigts. Puis le deuxième. La colle est froide aux doigts. Elle est longue ? Pas encore assez.</t>
+          <t>Le tiroir de papiers est entrouvert. Ça sent la colle, un peu sucré. Les volets laissent un rai mince. Le rai traverse la salle à manger. Il est fin, maman. Tu le vois, sur la table ? Oui, jusqu'au bois. Un fil pend du buffet. Les ciseaux attendent sur le bois. La chaise a un fil qui dépasse. Sur le bois du tiroir, un éclat de tiroir luit. Il brille, papa ! Tu le vois, sur le tiroir ? Oui, près du papier. Mila touche l'éclat de tiroir, un instant. Le bois est lisse, un peu froid. Il est froid. Tu coupes, Mila ? Oui, maintenant. En ce moment, Mila prend les ciseaux. Les ciseaux font un petit cri. Le papier est rouge, un peu rêche. C'est pour toi, papa. Une guirlande. Jusqu'à la fenêtre ? Oui. Tout le chemin. Nino arrive, en chaussettes silencieuses. Il s'assoit près de la table. La chaise craque, un peu. Son ventre touche le bord du bois. Nino reste assis. Tu viens coller, debout ? Nino ne dit rien. Ses mains restent sur ses genoux. Je reste assis. Debout, maintenant ! Mila tire trop vite sur sa manche. Nino se retient au dossier. Le premier anneau se déchire. Oh. La colle tombe sur le bois. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Tu veux coller près de Nino ? Maman se baisse à sa hauteur. Il tient le papier, toi ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les volets laissent un rai de poussière d'or. Un tiroir de papiers est ouvert. Ça sent la colle, un peu sucré. Un fil pend du buffet. Une paire de ciseaux attend sur le bois. La chaise a un fil qui dépasse. Tu as vu le rai de soleil, Mila ? Il est tout fin. Oui. Il traverse la salle. En ce moment, Mila coupe un rectangle. Les ciseaux font un petit cri. Le papier est rouge et un peu rêche. C'est pour toi, papa. Une guirlande. Jusqu'à la fenêtre ? Oui. Tout le chemin. Nino arrive avec des chaussettes silencieuses. Nino a un corps plus rond. Mila a un corps plus mince. Mila ne commente pas le corps. Le corps n'est pas une blague. On joue. Nino, tu veux coller ? Oui. Ils collent le premier anneau. Le papier frotte entre les doigts. Puis le deuxième. La colle est froide aux doigts. Elle est longue ? Pas encore assez.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le tiroir de papiers est entrouvert. Ça sent la colle, un peu sucré. Les volets laissent un rai mince. Le rai traverse la salle à manger. Il est fin, maman. Tu le vois, sur la table ? Oui, jusqu'au bois. Un fil pend du buffet. Les ciseaux attendent sur le bois. La chaise a un fil qui dépasse. Sur le bois du tiroir, un &lt;emphasis level="moderate"&gt;éclat de tiroir&lt;/emphasis&gt; luit. Il brille, papa ! Tu le vois, sur le tiroir ? Oui, près du papier. Mila touche l'éclat de tiroir, un instant. Le bois est lisse, un peu froid. Il est froid. Tu coupes, Mila ? Oui, maintenant. En ce moment, Mila prend les ciseaux. Les ciseaux font un petit cri. Le papier est rouge, un peu rêche. C'est pour toi, papa. Une guirlande. Jusqu'à la fenêtre ? Oui. Tout le chemin. Nino arrive, en chaussettes silencieuses. Il s'assoit près de la table. La chaise craque, un peu. Son ventre touche le bord du bois. Nino reste assis. Tu viens coller, debout ? Nino ne dit rien. Ses mains restent sur ses genoux. Je reste assis. Debout, maintenant ! Mila tire trop vite sur sa manche. Nino se retient au dossier. Le premier anneau se déchire. Oh. La colle tombe sur le bois. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Tu veux coller près de Nino ? Maman se baisse à sa hauteur. Il tient le papier, toi ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Hugo et Noé sont au gymnase avec papa. Ils se passent un ballon souple. Noé a un &lt;emphasis&gt;corps&lt;/emphasis&gt; plus rond. Hugo a un corps plus mince. Papa dit : le corps n'est pas une blague. On joue ensemble. Hugo ne commente pas le corps. Il passe le ballon. Noé le rend. Ils rient du jeu, pas du corps. Papa dit : l'amitié ne dépend pas de la forme. On joue. Le corps n'est pas une blague. [pause]</t>
+          <t>Le tiroir de papiers est entrouvert. Ça sent la colle, un peu sucré. Les volets laissent un rai mince. Le rai traverse la salle à manger. Il est fin, maman. Tu le vois, sur la table ? Oui, jusqu'au bois. Un fil pend du buffet. Les ciseaux attendent sur le bois. La chaise a un fil qui dépasse. Sur le bois du tiroir, un &lt;emphasis&gt;éclat de tiroir&lt;/emphasis&gt; luit. Il brille, papa ! Tu le vois, sur le tiroir ? Oui, près du papier. Mila touche l'éclat de tiroir, un instant. Le bois est lisse, un peu froid. Il est froid. Tu coupes, Mila ? Oui, maintenant. En ce moment, Mila prend les ciseaux. Les ciseaux font un petit cri. Le papier est rouge, un peu rêche. C'est pour toi, papa. Une guirlande. Jusqu'à la fenêtre ? Oui. Tout le chemin. Nino arrive, en chaussettes silencieuses. Il s'assoit près de la table. La chaise craque, un peu. Son ventre touche le bord du bois. Nino reste assis. Tu viens coller, debout ? Nino ne dit rien. Ses mains restent sur ses genoux. Je reste assis. Debout, maintenant ! Mila tire trop vite sur sa manche. Nino se retient au dossier. Le premier anneau se déchire. Oh. La colle tombe sur le bois. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Tu veux coller près de Nino ? Maman se baisse à sa hauteur. Il tient le papier, toi ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>éclat de tiroir</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,41 +1321,67 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_guirlande_et_nino_debout_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les volets laissent un rai de poussière d'or.
-narrateur|Un tiroir de papiers est ouvert.
+          <t>narrateur|Le tiroir de papiers est entrouvert.
 narrateur|Ça sent la colle, un peu sucré.
+narrateur|Les volets laissent un rai mince.
+narrateur|Le rai traverse la salle à manger.
+enfant-f|Il est fin, maman.
+maman|Tu le vois, sur la table ?
+enfant-f|Oui, jusqu'au bois.
 narrateur|Un fil pend du buffet.
-narrateur|Une paire de ciseaux attend sur le bois.
+narrateur|Les ciseaux attendent sur le bois.
 narrateur|La chaise a un fil qui dépasse.
-papa|Tu as vu le rai de soleil, Mila ?
-enfant-f|Il est tout fin.
-papa|Oui.
-papa|Il traverse la salle.
-narrateur|En ce moment, Mila coupe un rectangle.
+narrateur|Sur le bois du tiroir, un éclat de tiroir luit.
+enfant-f|Il brille, papa !
+papa|Tu le vois, sur le tiroir ?
+enfant-f|Oui, près du papier.
+narrateur|Mila touche l'éclat de tiroir, un instant.
+narrateur|Le bois est lisse, un peu froid.
+enfant-f|Il est froid.
+maman|Tu coupes, Mila ?
+enfant-f|Oui, maintenant.
+narrateur|En ce moment, Mila prend les ciseaux.
 narrateur|Les ciseaux font un petit cri.
-narrateur|Le papier est rouge et un peu rêche.
+narrateur|Le papier est rouge, un peu rêche.
 enfant-f|C'est pour toi, papa.
 enfant-f|Une guirlande.
 papa|Jusqu'à la fenêtre ?
 enfant-f|Oui.
 enfant-f|Tout le chemin.
-narrateur|Nino arrive avec des chaussettes silencieuses.
-narrateur|Nino a un corps plus rond.
-narrateur|Mila a un corps plus mince.
-narrateur|Mila ne commente pas le corps.
-papa|Le corps n'est pas une blague.
-papa|On joue.
-enfant-f|Nino, tu veux coller ?
-copain|Oui.
-narrateur|Ils collent le premier anneau.
-narrateur|Le papier frotte entre les doigts.
-narrateur|Puis le deuxième.
-narrateur|La colle est froide aux doigts.
-enfant-f|Elle est longue ?
-papa|Pas encore assez.</t>
+narrateur|Nino arrive, en chaussettes silencieuses.
+narrateur|Il s'assoit près de la table.
+narrateur|La chaise craque, un peu.
+narrateur|Son ventre touche le bord du bois.
+narrateur|Nino reste assis.
+enfant-f|Tu viens coller, debout ?
+narrateur|Nino ne dit rien.
+narrateur|Ses mains restent sur ses genoux.
+copain|Je reste assis.
+enfant-f|Debout, maintenant !
+narrateur|Mila tire trop vite sur sa manche.
+narrateur|Nino se retient au dossier.
+narrateur|Le premier anneau se déchire.
+enfant-f|Oh.
+narrateur|La colle tombe sur le bois.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Les épaules de Mila tombent un peu.
+narrateur|Ça serre, dans son ventre.
+maman|Tu veux coller près de Nino ?
+narrateur|Maman se baisse à sa hauteur.
+papa|Il tient le papier, toi ?</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>tiroir,papier,colle</t>
         </is>
       </c>
     </row>
@@ -1387,12 +1413,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le corps n'est pas une blague. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le corps n'est pas une &lt;emphasis level="moderate"&gt;blague&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Hugo joue avec Noé. Que fait-on ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le corps n'est pas une &lt;emphasis&gt;blague&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1455,18 +1481,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1481,34 +1507,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>blague</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1517,23 +1547,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=on_colle_ensemble_sans_rire_du_corps; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1566,17 +1596,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Ils ajoutent des anneaux. Un anneau rouge se déchire. Oh. On le répare. Nino tient les deux bords. Mila met un point de colle. L'anneau redevient rond. Bravo, Mila. Tu as réparé. Vous jouez. La guirlande arrive au milieu. Elle pèse un peu, toute douce. Il manque encore un bout. Encore trois. Encore trois. Ils collent. Le papier fait un petit bruit. Un anneau jaune s'ajoute au rouge. Le jaune, c'est le soleil. Le rouge, c'est la fête. Papa tient un bout près du buffet. Mila tient l'autre bout. Nino pose le dernier anneau. La guirlande touche la fenêtre. Elle est arrivée. L'amitié ne dépend pas de la forme. On joue.</t>
+          <t>Mila veut le tirer vers la fenêtre. Debout, Nino ! Sa voix se mélange à la colle. Nino reste assis. Mila refuse de foncer. Elle referme la main. Tu t'assois près de lui ? Maman s'accroupit à la même hauteur. Mila pose un genou près de la chaise. Tu colles, assis ? Nino ne dit rien. Il pousse un rectangle vers elle. Oui. D'accord. Merci, Mila. Papa a vu les deux mains sur le papier. Le ventre de Mila se desserre. Les épaules se relèvent un peu. La colle est froide, Mila ? Un peu, maman. Mila s'assoit, enfin. Son ventre touche le bois, froid. Ils collent le deuxième anneau. Le papier frotte entre les doigts. Il est rêche. Le rouge aussi. Un anneau jaune s'ajoute au rouge. Le jaune, c'est le soleil. Le rouge, c'est la fête. Elle avance, la guirlande ? Oui, papa. La guirlande arrive au milieu. Elle pèse un peu, tiède. Il manque un bout, Mila ? Trois, maman. Trois. Ils collent, sans se presser. Le papier fait un petit bruit.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Ils ajoutent des anneaux. Un anneau rouge se déchire. Oh. On le répare. Nino tient les deux bords. Mila met un point de colle. L'anneau redevient rond. Bravo, Mila. Tu as réparé. Vous jouez. La guirlande arrive au milieu. Elle pèse un peu, toute douce. Il manque encore un bout. Encore trois. Encore trois. Ils collent. Le papier fait un petit bruit. Un anneau jaune s'ajoute au rouge. Le jaune, c'est le soleil. Le rouge, c'est la fête. Papa tient un bout près du buffet. Mila tient l'autre bout. Nino pose le dernier anneau. La guirlande touche la fenêtre. Elle est arrivée. L'amitié ne dépend pas de la forme. On joue.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila veut le tirer vers la fenêtre. Debout, Nino ! Sa voix se mélange à la colle. Nino reste assis. Mila refuse de foncer. Elle referme la main. Tu t'assois près de lui ? Maman s'accroupit à la même hauteur. Mila pose un genou près de la chaise. Tu colles, assis ? Nino ne dit rien. Il pousse un rectangle vers elle. Oui. &lt;emphasis level="moderate"&gt;D'accord&lt;/emphasis&gt;. Merci, Mila. Papa a vu les deux mains sur le papier. Le ventre de Mila se desserre. Les épaules se relèvent un peu. La colle est froide, Mila ? Un peu, maman. Mila s'assoit, enfin. Son ventre touche le bois, froid. Ils collent le deuxième anneau. Le papier frotte entre les doigts. Il est rêche. Le rouge aussi. Un anneau jaune s'ajoute au rouge. Le jaune, c'est le soleil. Le rouge, c'est la fête. Elle avance, la guirlande ? Oui, papa. La guirlande arrive au milieu. Elle pèse un peu, tiède. Il manque un bout, Mila ? Trois, maman. Trois. Ils collent, sans se presser. Le papier fait un petit bruit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Hugo a joué avec Noé. Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'était pas une blague. [pause]</t>
+          <t>Mila veut le tirer vers la fenêtre. Debout, Nino ! Sa voix se mélange à la colle. Nino reste assis. Mila refuse de foncer. Elle referme la main. Tu t'assois près de lui ? Maman s'accroupit à la même hauteur. Mila pose un genou près de la chaise. Tu colles, assis ? Nino ne dit rien. Il pousse un rectangle vers elle. Oui. &lt;emphasis&gt;D'accord&lt;/emphasis&gt;. Merci, Mila. Papa a vu les deux mains sur le papier. Le ventre de Mila se desserre. Les épaules se relèvent un peu. La colle est froide, Mila ? Un peu, maman. Mila s'assoit, enfin. Son ventre touche le bois, froid. Ils collent le deuxième anneau. Le papier frotte entre les doigts. Il est rêche. Le rouge aussi. Un anneau jaune s'ajoute au rouge. Le jaune, c'est le soleil. Le rouge, c'est la fête. Elle avance, la guirlande ? Oui, papa. La guirlande arrive au milieu. Elle pèse un peu, tiède. Il manque un bout, Mila ? Trois, maman. Trois. Ils collent, sans se presser. Le papier fait un petit bruit. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1623,7 +1653,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1631,10 +1661,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1657,30 +1687,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>D'accord</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1689,10 +1719,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1705,38 +1735,54 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_s_assoit_attend_le_silence_dit_d_accord; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Ils ajoutent des anneaux.
-narrateur|Un anneau rouge se déchire.
-enfant-f|Oh.
-copain|On le répare.
-narrateur|Nino tient les deux bords.
-narrateur|Mila met un point de colle.
-narrateur|L'anneau redevient rond.
-papa|Bravo, Mila.
-papa|Tu as réparé.
-papa|Vous jouez.
-narrateur|La guirlande arrive au milieu.
-narrateur|Elle pèse un peu, toute douce.
-narrateur|Il manque encore un bout.
-enfant-f|Encore trois.
-copain|Encore trois.
-narrateur|Ils collent.
-narrateur|Le papier fait un petit bruit.
+          <t>narrateur|Mila veut le tirer vers la fenêtre.
+enfant-f|Debout, Nino !
+narrateur|Sa voix se mélange à la colle.
+narrateur|Nino reste assis.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la main.
+maman|Tu t'assois près de lui ?
+narrateur|Maman s'accroupit à la même hauteur.
+narrateur|Mila pose un genou près de la chaise.
+enfant-f|Tu colles, assis ?
+narrateur|Nino ne dit rien.
+narrateur|Il pousse un rectangle vers elle.
+copain|Oui.
+enfant-f|D'accord.
+papa|Merci, Mila.
+narrateur|Papa a vu les deux mains sur le papier.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|La colle est froide, Mila ?
+enfant-f|Un peu, maman.
+narrateur|Mila s'assoit, enfin.
+narrateur|Son ventre touche le bois, froid.
+narrateur|Ils collent le deuxième anneau.
+narrateur|Le papier frotte entre les doigts.
+enfant-f|Il est rêche.
+copain|Le rouge aussi.
 narrateur|Un anneau jaune s'ajoute au rouge.
 enfant-f|Le jaune, c'est le soleil.
 copain|Le rouge, c'est la fête.
-narrateur|Papa tient un bout près du buffet.
-narrateur|Mila tient l'autre bout.
-narrateur|Nino pose le dernier anneau.
-narrateur|La guirlande touche la fenêtre.
-enfant-f|Elle est arrivée.
-papa|L'amitié ne dépend pas de la forme.
-papa|On joue.</t>
+papa|Elle avance, la guirlande ?
+enfant-f|Oui, papa.
+narrateur|La guirlande arrive au milieu.
+narrateur|Elle pèse un peu, tiède.
+maman|Il manque un bout, Mila ?
+enfant-f|Trois, maman.
+copain|Trois.
+narrateur|Ils collent, sans se presser.
+narrateur|Le papier fait un petit bruit.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>papier,colle</t>
         </is>
       </c>
     </row>
@@ -1763,17 +1809,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On la regarde un moment ? Oui. Le rai de soleil traverse un anneau. Le rouge devient plus clair. Il brille. C'est ton cadeau. Merci. Tu as fini de coller ? Oui, papa. Ils essuient la colle sur le torchon. Le torchon devient un peu dur. Le tiroir se referme. La salle sent encore le papier. Plus tard, le gâteau. Merci, Nino. Merci, Mila.</t>
+          <t>Mila se lève trop vite. Jusqu'à la fenêtre, d'un coup ! Elle tire Nino vers le haut. Nino reste collé à la chaise. Attends. Je la tends ! La guirlande penche vers le buffet. Un anneau rouge se fend, presque. Ça tombe ! Mila veut rattraper le fil, d'un coup. Mila refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde le tiroir, elle écoute la salle. Sur le bois du tiroir, un éclat de tiroir luit. Là, près du papier. Tu le vois, toi ? Oui, papa. Mila baisse la guirlande, sans se presser. Nino tient un bout, assis. Moi, près de la fenêtre. Vous tenez les deux bouts ? Oui, maman. Moi, le bas. Papa tient un bout près du buffet. La guirlande touche la fenêtre. Elle est arrivée. On la regarde un moment ? Oui. Le rai traverse un anneau rouge. Il brille. C'est ton cadeau.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On la regarde un moment ? Oui. Le rai de soleil traverse un anneau. Le rouge devient plus clair. Il brille. C'est ton cadeau. Merci. Tu as fini de coller ? Oui, papa. Ils essuient la colle sur le torchon. Le torchon devient un peu dur. Le tiroir se referme. La salle sent encore le papier. Plus tard, le gâteau. Merci, Nino. Merci, Mila.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila se lève trop vite. Jusqu'à la fenêtre, d'un coup ! Elle tire Nino vers le haut. Nino reste collé à la chaise. Attends. Je la tends ! La guirlande penche vers le buffet. Un anneau rouge se fend, presque. Ça tombe ! Mila veut rattraper le fil, d'un coup. Mila refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde le tiroir, elle écoute la salle. Sur le bois du tiroir, un &lt;emphasis level="moderate"&gt;éclat de tiroir&lt;/emphasis&gt; luit. Là, près du papier. Tu le vois, toi ? Oui, papa. Mila baisse la guirlande, sans se presser. Nino tient un bout, assis. Moi, près de la fenêtre. Vous tenez les deux bouts ? Oui, maman. Moi, le bas. Papa tient un bout près du buffet. La guirlande touche la fenêtre. Elle est arrivée. On la regarde un moment ? Oui. Le rai traverse un anneau rouge. Il brille. C'est ton cadeau.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa range le ballon. Hugo essuie ses &lt;emphasis&gt;main&lt;/emphasis&gt;s. [pause]</t>
+          <t>&lt;low-pitch&gt;Mila se lève trop vite. Jusqu'à la fenêtre, d'un coup ! Elle tire Nino vers le haut. Nino reste collé à la chaise. Attends. Je la tends ! La guirlande penche vers le buffet. Un anneau rouge se fend, presque. Ça tombe ! Mila veut rattraper le fil, d'un coup. Mila refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde le tiroir, elle écoute la salle. Sur le bois du tiroir, un &lt;emphasis&gt;éclat de tiroir&lt;/emphasis&gt; luit. Là, près du papier. Tu le vois, toi ? Oui, papa. Mila baisse la guirlande, sans se presser. Nino tient un bout, assis. Moi, près de la fenêtre. Vous tenez les deux bouts ? Oui, maman. Moi, le bas. Papa tient un bout près du buffet. La guirlande touche la fenêtre. Elle est arrivée. On la regarde un moment ? Oui. Le rai traverse un anneau rouge. Il brille. C'est ton cadeau.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1820,7 +1866,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1828,22 +1874,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1854,30 +1904,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de tiroir</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1886,39 +1936,65 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat_de_tiroir; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>papa|On la regarde un moment ?
+          <t>narrateur|Mila se lève trop vite.
+enfant-f|Jusqu'à la fenêtre, d'un coup !
+narrateur|Elle tire Nino vers le haut.
+narrateur|Nino reste collé à la chaise.
+copain|Attends.
+enfant-f|Je la tends !
+narrateur|La guirlande penche vers le buffet.
+narrateur|Un anneau rouge se fend, presque.
+enfant-f|Ça tombe !
+narrateur|Mila veut rattraper le fil, d'un coup.
+narrateur|Mila refuse de foncer, cette fois.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape fort, dans sa poitrine.
+narrateur|Personne ne dit la suite à voix haute.
+narrateur|Elle regarde le tiroir, elle écoute la salle.
+narrateur|Sur le bois du tiroir, un éclat de tiroir luit.
+enfant-f|Là, près du papier.
+papa|Tu le vois, toi ?
+enfant-f|Oui, papa.
+narrateur|Mila baisse la guirlande, sans se presser.
+narrateur|Nino tient un bout, assis.
+enfant-f|Moi, près de la fenêtre.
+maman|Vous tenez les deux bouts ?
+enfant-f|Oui, maman.
+copain|Moi, le bas.
+narrateur|Papa tient un bout près du buffet.
+narrateur|La guirlande touche la fenêtre.
+enfant-f|Elle est arrivée.
+papa|On la regarde un moment ?
 enfant-f|Oui.
-narrateur|Le rai de soleil traverse un anneau.
-narrateur|Le rouge devient plus clair.
+narrateur|Le rai traverse un anneau rouge.
 copain|Il brille.
-enfant-f|C'est ton cadeau.
-papa|Merci.
-papa|Tu as fini de coller ?
-enfant-f|Oui, papa.
-narrateur|Ils essuient la colle sur le torchon.
-narrateur|Le torchon devient un peu dur.
-narrateur|Le tiroir se referme.
-narrateur|La salle sent encore le papier.
-papa|Plus tard, le gâteau.
-enfant-f|Merci, Nino.
-copain|Merci, Mila.</t>
+enfant-f|C'est ton cadeau.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>papier,fenêtre</t>
         </is>
       </c>
     </row>
@@ -1945,17 +2021,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>On a tendu la guirlande. Jusqu'à la fenêtre. Vous avez joué. Le rai de soleil reste dans le rouge.</t>
+          <t>Le tiroir brillait, papa. Tu le vois, comme tout à l'heure ? Oui, sur le tiroir. Ils essuient la colle sur le torchon. Le torchon devient un peu dur. On le laisse près de nous ? Oui, maman. Ça sentait la colle. Le tiroir est là. Le tiroir se referme, un peu. Mila respire, plus large. On reste un peu ? Oui. Plus tard, le gâteau ? Oui, papa. Les joues de Mila se réchauffent. Les ciseaux restent tièdes sous la main. Le rai a glissé sur la table. Il est pâle. Comme tout à l'heure ? Oui, maman. Le fil pend, toi ? Un peu, papa. La chaise ne craque plus. Elle est tiède. On la laisse à table ? Oui. Un éclat de tiroir reste pâle. Le rouge garde un rai mince.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>On a tendu la guirlande. Jusqu'à la fenêtre. Vous avez joué. Le rai de soleil reste dans le rouge.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le tiroir brillait, papa. Tu le vois, comme tout à l'heure ? Oui, sur le tiroir. Ils essuient la colle sur le torchon. Le torchon devient un peu dur. On le laisse près de nous ? Oui, maman. Ça sentait la colle. Le tiroir est là. Le tiroir se referme, un peu. Mila respire, plus large. On reste un peu ? Oui. Plus tard, le gâteau ? Oui, papa. Les joues de Mila se réchauffent. Les ciseaux restent tièdes sous la main. Le rai a glissé sur la table. Il est pâle. Comme tout à l'heure ? Oui, maman. Le fil pend, toi ? Un peu, papa. La chaise ne craque plus. Elle est tiède. On la laisse à table ? Oui. Un &lt;emphasis level="moderate"&gt;éclat de tiroir&lt;/emphasis&gt; reste pâle. Le rouge garde un rai mince.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le tiroir brillait, papa. Tu le vois, comme tout à l'heure ? Oui, sur le tiroir. Ils essuient la colle sur le torchon. Le torchon devient un peu dur. On le laisse près de nous ? Oui, maman. Ça sentait la colle. Le tiroir est là. Le tiroir se referme, un peu. Mila respire, plus large. On reste un peu ? Oui. Plus tard, le gâteau ? Oui, papa. Les joues de Mila se réchauffent. Les ciseaux restent tièdes sous la main. Le rai a glissé sur la table. Il est pâle. Comme tout à l'heure ? Oui, maman. Le fil pend, toi ? Un peu, papa. La chaise ne craque plus. Elle est tiède. On la laisse à table ? Oui. Un &lt;emphasis&gt;éclat de tiroir&lt;/emphasis&gt; reste pâle. Le rouge garde un rai mince.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2002,7 +2078,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2010,10 +2086,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.12</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2022,12 +2098,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2036,17 +2112,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de tiroir</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2055,11 +2135,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2068,27 +2148,61 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_tiroir_reste_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|On a tendu la guirlande.
-copain|Jusqu'à la fenêtre.
-papa|Vous avez joué.
-narrateur|Le rai de soleil reste dans le rouge.</t>
+          <t>enfant-f|Le tiroir brillait, papa.
+papa|Tu le vois, comme tout à l'heure ?
+enfant-f|Oui, sur le tiroir.
+narrateur|Ils essuient la colle sur le torchon.
+narrateur|Le torchon devient un peu dur.
+maman|On le laisse près de nous ?
+enfant-f|Oui, maman.
+enfant-f|Ça sentait la colle.
+maman|Le tiroir est là.
+narrateur|Le tiroir se referme, un peu.
+narrateur|Mila respire, plus large.
+papa|On reste un peu ?
+enfant-f|Oui.
+papa|Plus tard, le gâteau ?
+enfant-f|Oui, papa.
+narrateur|Les joues de Mila se réchauffent.
+narrateur|Les ciseaux restent tièdes sous la main.
+narrateur|Le rai a glissé sur la table.
+enfant-f|Il est pâle.
+maman|Comme tout à l'heure ?
+enfant-f|Oui, maman.
+papa|Le fil pend, toi ?
+enfant-f|Un peu, papa.
+narrateur|La chaise ne craque plus.
+enfant-f|Elle est tiède.
+maman|On la laisse à table ?
+enfant-f|Oui.
+narrateur|Un éclat de tiroir reste pâle.
+narrateur|Le rouge garde un rai mince.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>salle</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2194,6 +2308,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>